<commit_message>
modify program code etc
</commit_message>
<xml_diff>
--- a/Reference/バーコード現品票20260402/ボディー　バーコード一覧.xlsx
+++ b/Reference/バーコード現品票20260402/ボディー　バーコード一覧.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\myProgram\GitHub\body_inspect_visualize_coba\Reference\バーコード現品票20260402\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B836245-D6A3-4A6B-B16D-815D8C746F93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA5BE2C-0DE0-4AE1-AA07-47C04BF7B507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4A0C8197-23CB-4D59-8779-3CDAF6BEF46B}"/>
   </bookViews>
@@ -241,7 +241,7 @@
       <charset val="128"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -251,12 +251,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -378,7 +372,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -831,15 +825,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>32302</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>32712</xdr:rowOff>
+      <xdr:colOff>24020</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>40994</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2030302</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>644712</xdr:rowOff>
+      <xdr:colOff>2022020</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>652994</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -869,7 +863,7 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="719759" y="6136995"/>
+          <a:off x="711477" y="5474385"/>
           <a:ext cx="1998000" cy="612000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1560,62 +1554,6 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>32302</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>32555</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1998000" cy="612000"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="21" name="図 20">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A5AD845B-9491-4682-8F49-1A923E7F241C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="719759" y="5465946"/>
-          <a:ext cx="1998000" cy="612000"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>4</xdr:col>
@@ -2272,7 +2210,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="52.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
       <c r="B8" s="10"/>

</xml_diff>